<commit_message>
Copy pass on the 16 laddbox descriptions (best-practice sharpening)
Sharpened the vague/redundant box subtitles to concrete, differentiated
one-liners; kept the already-strong concrete ones (no change-for-change,
no fabricated specs): Zaptec Go → "Kompakt, upp till 22 kW"; Zaptec Go 2 →
"Nu med inbyggd skärm"; Easee → "Smart laddning via app"; Tesla Wall
Connector → "Fast kabel, 7,3 m"; Defa → "Display, klarar −40 °C"; Zaptec Pro
→ dropped redundant "· offert" (badge already says Offert).

Applied to data.js + build_xlsx.py + verify_faithful.py EXPECTED; .xlsx
regenerated with xlsxwriter; oracle PASS (deep-equal). Verified in preview.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/laddbox-kalkylator-data.xlsx
+++ b/excel/laddbox-kalkylator-data.xlsx
@@ -149,7 +149,7 @@
     <t>Zaptec Go</t>
   </si>
   <si>
-    <t>Kompakt favorit</t>
+    <t>Kompakt, upp till 22 kW</t>
   </si>
   <si>
     <t>Bästsäljare</t>
@@ -167,7 +167,7 @@
     <t>Zaptec Go 2</t>
   </si>
   <si>
-    <t>Inbyggd display</t>
+    <t>Nu med inbyggd skärm</t>
   </si>
   <si>
     <t>Rekommenderas</t>
@@ -182,7 +182,7 @@
     <t>Easee Charge Up</t>
   </si>
   <si>
-    <t>Smart &amp; nätt</t>
+    <t>Smart laddning via app</t>
   </si>
   <si>
     <t>https://ampy.se/laddboxar/easee-charge-up/</t>
@@ -221,7 +221,7 @@
     <t>Tesla Wall Connector</t>
   </si>
   <si>
-    <t>Fast kabel 7,3 m</t>
+    <t>Fast kabel, 7,3 m</t>
   </si>
   <si>
     <t>https://ampy.se/laddboxar/tesla-wall-connector/</t>
@@ -284,7 +284,7 @@
     <t>Defa Power</t>
   </si>
   <si>
-    <t>Display &amp; −40 °C</t>
+    <t>Display, klarar −40 °C</t>
   </si>
   <si>
     <t>https://ampy.se/laddboxar/defa-power/</t>
@@ -332,7 +332,7 @@
     <t>Zaptec Pro</t>
   </si>
   <si>
-    <t>Skalbar för flera platser · offert</t>
+    <t>Skalbar för flera platser</t>
   </si>
   <si>
     <t>Offert</t>

</xml_diff>